<commit_message>
Cambio de PARAMETROS a parametros.py para fechas
</commit_message>
<xml_diff>
--- a/data/PARAMETROS.xlsx
+++ b/data/PARAMETROS.xlsx
@@ -8,21 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\MATINAL ONLINE\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9DBD292-5803-43F7-A2B8-EBA9AC6CB7B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF8DCC87-B939-48E8-B124-1177FDC02E7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C4405403-8AD1-46BC-9444-73E3B4DA109B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C4405403-8AD1-46BC-9444-73E3B4DA109B}"/>
   </bookViews>
   <sheets>
-    <sheet name="FECHAS" sheetId="1" r:id="rId1"/>
-    <sheet name="MARCAS" sheetId="4" r:id="rId2"/>
-    <sheet name="SEGMENTOS" sheetId="5" r:id="rId3"/>
-    <sheet name="VENDEDORES" sheetId="2" r:id="rId4"/>
-    <sheet name="INVENDIBLE" sheetId="3" r:id="rId5"/>
-    <sheet name="CCC" sheetId="6" r:id="rId6"/>
+    <sheet name="MARCAS" sheetId="4" r:id="rId1"/>
+    <sheet name="SEGMENTOS" sheetId="5" r:id="rId2"/>
+    <sheet name="VENDEDORES" sheetId="2" r:id="rId3"/>
+    <sheet name="INVENDIBLE" sheetId="3" r:id="rId4"/>
+    <sheet name="CCC" sheetId="6" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="DatosExternos_1" localSheetId="5" hidden="1">'CCC'!$A$2:$A$6</definedName>
-    <definedName name="DatosExternos_1" localSheetId="0" hidden="1">FECHAS!#REF!</definedName>
+    <definedName name="DatosExternos_1" localSheetId="4" hidden="1">'CCC'!$A$2:$A$6</definedName>
     <definedName name="DiaLimiteLiquidacion">#REF!</definedName>
     <definedName name="FechaHoy">#REF!</definedName>
     <definedName name="MesOperativoFin">#REF!</definedName>
@@ -75,10 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4294963687" uniqueCount="76">
-  <si>
-    <t>TABLAS de PARAMETROS</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="68">
   <si>
     <t>VENDEDORES</t>
   </si>
@@ -86,12 +81,6 @@
     <t>INVENDIBLE</t>
   </si>
   <si>
-    <t>PARAMETRO</t>
-  </si>
-  <si>
-    <t>VALOR</t>
-  </si>
-  <si>
     <t>CodVend</t>
   </si>
   <si>
@@ -116,34 +105,19 @@
     <t>Hasta</t>
   </si>
   <si>
-    <t>Año</t>
-  </si>
-  <si>
     <t>GALARZA, MARCELA VIRGINIA</t>
   </si>
   <si>
-    <t>Mes</t>
-  </si>
-  <si>
     <t>PATERNOSTER, LEANDRO</t>
   </si>
   <si>
-    <t>Dia Matinal</t>
-  </si>
-  <si>
     <t>RODRIGUEZ, CRISTIAN</t>
   </si>
   <si>
-    <t>Dia Venta</t>
-  </si>
-  <si>
     <t>OLMOS, JONATAN</t>
   </si>
   <si>
     <t>OBJETIVOS POR MARCA</t>
-  </si>
-  <si>
-    <t>Dia Anterior</t>
   </si>
   <si>
     <t>FUMAROLA, ANGEL</t>
@@ -312,7 +286,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -331,22 +305,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="24"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -524,76 +482,59 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="7" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="4" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -603,146 +544,7 @@
     <cellStyle name="Porcentaje" xfId="2" builtinId="5"/>
     <cellStyle name="Porcentaje 3" xfId="3" xr:uid="{43E87D2C-7C1D-4FA2-8AA7-FD8C1DFF4CD5}"/>
   </cellStyles>
-  <dxfs count="28">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="mediumDashed">
-          <color auto="1"/>
-        </left>
-        <right style="mediumDashed">
-          <color auto="1"/>
-        </right>
-        <top style="mediumDashed">
-          <color auto="1"/>
-        </top>
-        <bottom style="mediumDashed">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="13" formatCode="0%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="mediumDashed">
-          <color auto="1"/>
-        </left>
-        <right style="mediumDashed">
-          <color auto="1"/>
-        </right>
-        <top style="mediumDashed">
-          <color auto="1"/>
-        </top>
-        <bottom style="mediumDashed">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal style="mediumDashed">
-          <color auto="1"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="mediumDashed">
-          <color auto="1"/>
-        </top>
-        <bottom style="mediumDashed">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <border outline="0">
-        <left style="mediumDashed">
-          <color auto="1"/>
-        </left>
-        <right style="mediumDashed">
-          <color auto="1"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="mediumDashed">
-          <color auto="1"/>
-        </top>
-        <bottom style="mediumDashed">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <border outline="0">
-        <right style="mediumDashed">
-          <color auto="1"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="25">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1216,7 +1018,7 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -1226,29 +1028,121 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color rgb="FF000000"/>
+        <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="mediumDashed">
+          <color auto="1"/>
+        </left>
+        <right style="mediumDashed">
+          <color auto="1"/>
+        </right>
+        <top style="mediumDashed">
+          <color auto="1"/>
+        </top>
+        <bottom style="mediumDashed">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="13" formatCode="0%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="mediumDashed">
+          <color auto="1"/>
+        </left>
+        <right style="mediumDashed">
+          <color auto="1"/>
+        </right>
+        <top style="mediumDashed">
+          <color auto="1"/>
+        </top>
+        <bottom style="mediumDashed">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal style="mediumDashed">
+          <color auto="1"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="mediumDashed">
+          <color auto="1"/>
+        </top>
+        <bottom style="mediumDashed">
+          <color auto="1"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
         <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
       </font>
+      <border outline="0">
+        <left style="mediumDashed">
+          <color auto="1"/>
+        </left>
+        <right style="mediumDashed">
+          <color auto="1"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="mediumDashed">
+          <color auto="1"/>
+        </top>
+        <bottom style="mediumDashed">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <border outline="0">
+        <right style="mediumDashed">
+          <color auto="1"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
@@ -1279,21 +1173,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{026C9EB2-DFAD-4F3F-8261-D379BAB65AB3}" name="FECHAS" displayName="FECHAS" ref="A4:B9" totalsRowShown="0" headerRowDxfId="27">
-  <autoFilter ref="A4:B9" xr:uid="{A722C27F-65BA-409E-948F-01EB13F8EDB1}">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{5F8EB6F8-D34A-4F96-B2CB-CE97A0A5AF76}" name="PARAMETRO" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{02ADF40C-84AB-4893-A09B-4990ECAA5EE4}" name="VALOR"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{CC75DCDA-A932-4B50-BF5F-C320E376D186}" name="MARCAS" displayName="MARCAS" ref="A2:F11" totalsRowShown="0" headerRowDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{CC75DCDA-A932-4B50-BF5F-C320E376D186}" name="MARCAS" displayName="MARCAS" ref="A2:F11" totalsRowShown="0" headerRowDxfId="24">
   <autoFilter ref="A2:F11" xr:uid="{CC75DCDA-A932-4B50-BF5F-C320E376D186}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1303,64 +1183,64 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{3B1E40F3-B52B-4F83-9864-1E305078DDA7}" name="Marca" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{AF4E0D6F-D9EC-4A8B-8934-A6FEC54D4113}" name="OBJ" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{57E7D2FF-72CF-4BBD-8A29-52A636F1059E}" name="CEBE" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{ED003413-B75E-4DFB-A39C-F0B86E72FD67}" name="GROSS" dataDxfId="2" dataCellStyle="Moneda"/>
-    <tableColumn id="5" xr3:uid="{ACC8A0FD-DDE0-4020-AE4F-E6CD410527BD}" name="Porc_Requerido" dataDxfId="1" dataCellStyle="Porcentaje"/>
-    <tableColumn id="6" xr3:uid="{4A683FD4-D28C-44F8-8661-FA19D29705F5}" name="Obj_Cobertura" dataDxfId="0" dataCellStyle="Porcentaje"/>
+    <tableColumn id="1" xr3:uid="{3B1E40F3-B52B-4F83-9864-1E305078DDA7}" name="Marca" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{AF4E0D6F-D9EC-4A8B-8934-A6FEC54D4113}" name="OBJ" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{57E7D2FF-72CF-4BBD-8A29-52A636F1059E}" name="CEBE" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{ED003413-B75E-4DFB-A39C-F0B86E72FD67}" name="GROSS" dataDxfId="20" dataCellStyle="Moneda"/>
+    <tableColumn id="5" xr3:uid="{ACC8A0FD-DDE0-4020-AE4F-E6CD410527BD}" name="Porc_Requerido" dataDxfId="19" dataCellStyle="Porcentaje"/>
+    <tableColumn id="6" xr3:uid="{4A683FD4-D28C-44F8-8661-FA19D29705F5}" name="Obj_Cobertura" dataDxfId="18" dataCellStyle="Porcentaje"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{E533F54E-6DD8-48BE-91C6-748C1A4C632A}" name="SEGMENTOS" displayName="SEGMENTOS" ref="A2:C7" totalsRowShown="0">
   <autoFilter ref="A2:C7" xr:uid="{E533F54E-6DD8-48BE-91C6-748C1A4C632A}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{42157F4C-5146-4258-9A27-F96869134E1F}" name="SEGMENTO" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{7FFE5579-826E-4C3A-A8D6-70B07D3913C5}" name="OBJ" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{A88CCE33-16B2-45F9-98C8-D66F3170B5F3}" name="Porc_Requerido" dataDxfId="23" dataCellStyle="Porcentaje"/>
+    <tableColumn id="1" xr3:uid="{42157F4C-5146-4258-9A27-F96869134E1F}" name="SEGMENTO" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{7FFE5579-826E-4C3A-A8D6-70B07D3913C5}" name="OBJ" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{A88CCE33-16B2-45F9-98C8-D66F3170B5F3}" name="Porc_Requerido" dataDxfId="15" dataCellStyle="Porcentaje"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{C7FD53BB-ACC2-4621-BBB4-4D1A0E3D37AC}" name="VENDEDORES" displayName="VENDEDORES" ref="A2:D27" totalsRowShown="0" headerRowDxfId="22" headerRowBorderDxfId="21" tableBorderDxfId="20" totalsRowBorderDxfId="19">
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{C7FD53BB-ACC2-4621-BBB4-4D1A0E3D37AC}" name="VENDEDORES" displayName="VENDEDORES" ref="A2:D27" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="13" tableBorderDxfId="12" totalsRowBorderDxfId="11">
   <autoFilter ref="A2:D27" xr:uid="{C7FD53BB-ACC2-4621-BBB4-4D1A0E3D37AC}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{DB3F861C-B76A-412C-9F75-A11FB6A69AE3}" name="CodVend" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{97DC079F-58B4-4136-80A8-F1E4423750E9}" name="Nombre" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{0C09E09E-73B1-48EB-9A0A-DA935FA7EF2E}" name="SUP" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{3D0816F0-3BD3-4F31-99E7-BB7DA2335E96}" name="Rutas" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{DB3F861C-B76A-412C-9F75-A11FB6A69AE3}" name="CodVend" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{97DC079F-58B4-4136-80A8-F1E4423750E9}" name="Nombre" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{0C09E09E-73B1-48EB-9A0A-DA935FA7EF2E}" name="SUP" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{3D0816F0-3BD3-4F31-99E7-BB7DA2335E96}" name="Rutas" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{486E829A-C8F9-4626-A894-C7D14E4BEBAF}" name="INVENDIBLE" displayName="INVENDIBLE" ref="A2:D4" totalsRowShown="0">
   <autoFilter ref="A2:D4" xr:uid="{486E829A-C8F9-4626-A894-C7D14E4BEBAF}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{5F5C4ED6-C81C-4F03-BFF4-CDF18856D769}" name="COD" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{4EAD7D8A-BE80-4C7A-AB3C-FD5BB7DB4DA2}" name="DESCRIPCION" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{03A150D1-B2A3-4FD2-BA8E-9C4CD55F8160}" name="Desde" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{20D44A67-0879-443C-80A2-B2A6D60A4752}" name="Hasta" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{5F5C4ED6-C81C-4F03-BFF4-CDF18856D769}" name="COD" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{4EAD7D8A-BE80-4C7A-AB3C-FD5BB7DB4DA2}" name="DESCRIPCION" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{03A150D1-B2A3-4FD2-BA8E-9C4CD55F8160}" name="Desde" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{20D44A67-0879-443C-80A2-B2A6D60A4752}" name="Hasta" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{F022A723-E976-4010-B123-8739FF36BC55}" name="CCC" displayName="CCC" ref="A2:B6" tableType="queryTable" totalsRowShown="0" headerRowDxfId="10">
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{F022A723-E976-4010-B123-8739FF36BC55}" name="CCC" displayName="CCC" ref="A2:B6" tableType="queryTable" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A2:B6" xr:uid="{F022A723-E976-4010-B123-8739FF36BC55}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{F9712261-341A-4566-B58B-C6D6BD113E8E}" uniqueName="1" name="Taxonomia" queryTableFieldId="1" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{9A19E11C-0E07-48DF-8026-BCF521E046F1}" uniqueName="3" name="OBJ_PEPSICO" queryTableFieldId="3" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{F9712261-341A-4566-B58B-C6D6BD113E8E}" uniqueName="1" name="Taxonomia" queryTableFieldId="1" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{9A19E11C-0E07-48DF-8026-BCF521E046F1}" uniqueName="3" name="OBJ_PEPSICO" queryTableFieldId="3" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1658,90 +1538,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3186E597-93DB-4F18-9E0E-C567C6FCC43D}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="13.77734375" customWidth="1"/>
-    <col min="2" max="2" width="11.5546875" customWidth="1"/>
-    <col min="3" max="3" width="11.88671875" customWidth="1"/>
-    <col min="4" max="16384" width="11.5546875" hidden="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" ht="31.2" x14ac:dyDescent="0.6">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="3"/>
-    </row>
-    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="10">
-        <f>YEAR(B8)</f>
-        <v>2026</v>
-      </c>
-      <c r="C5" s="10"/>
-    </row>
-    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="16">
-        <v>8</v>
-      </c>
-      <c r="C6" s="17"/>
-    </row>
-    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="21">
-        <v>46265</v>
-      </c>
-      <c r="C7" s="22"/>
-    </row>
-    <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="21">
-        <v>46263</v>
-      </c>
-      <c r="C8" s="22"/>
-    </row>
-    <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="21">
-        <v>46262</v>
-      </c>
-      <c r="C9" s="22"/>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="C8:C9">
-    <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
-      <formula>"Ingresar Dia Matinal"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D6D016D-89A0-46E5-B1CB-1AE10E233483}">
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1752,212 +1548,212 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>21</v>
+      <c r="A1" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="10" t="s">
+      <c r="A2" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="16">
+        <v>15500</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="17">
+        <v>376482.3</v>
+      </c>
+      <c r="E3" s="18">
+        <v>1.06</v>
+      </c>
+      <c r="F3" s="18">
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" s="10" t="s">
+      <c r="B4" s="16">
+        <v>11300</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="17">
+        <v>288925</v>
+      </c>
+      <c r="E4" s="18">
+        <v>1.06</v>
+      </c>
+      <c r="F4" s="18">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="F2" s="10" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="23">
-        <v>15500</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="B5" s="16">
+        <v>4800</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="17">
+        <v>120118.7</v>
+      </c>
+      <c r="E5" s="18">
+        <v>1.06</v>
+      </c>
+      <c r="F5" s="18">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="16">
+        <v>3500</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="17">
+        <v>86280</v>
+      </c>
+      <c r="E6" s="18">
+        <v>1.06</v>
+      </c>
+      <c r="F6" s="18">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="24">
-        <v>376482.3</v>
-      </c>
-      <c r="E3" s="25">
+      <c r="B7" s="16">
+        <v>6800</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="17">
+        <v>111618.7</v>
+      </c>
+      <c r="E7" s="18">
         <v>1.06</v>
       </c>
-      <c r="F3" s="25">
-        <v>0.89</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="F7" s="18">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="23">
-        <v>11300</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D4" s="24">
-        <v>288925</v>
-      </c>
-      <c r="E4" s="25">
+      <c r="B8" s="16">
+        <v>14400</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="17">
+        <v>212003.3</v>
+      </c>
+      <c r="E8" s="18">
         <v>1.06</v>
       </c>
-      <c r="F4" s="25">
-        <v>0.85</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="F8" s="18">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="23">
-        <v>4800</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" s="24">
-        <v>120118.7</v>
-      </c>
-      <c r="E5" s="25">
+      <c r="B9" s="16">
+        <v>5800</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="17">
+        <v>133612.6</v>
+      </c>
+      <c r="E9" s="18">
         <v>1.06</v>
       </c>
-      <c r="F5" s="25">
-        <v>0.66</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="23">
-        <v>3500</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" s="24">
-        <v>86280</v>
-      </c>
-      <c r="E6" s="25">
+      <c r="F9" s="18">
+        <v>0.56000000000000005</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="16">
+        <v>500</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="17">
+        <v>10727.7</v>
+      </c>
+      <c r="E10" s="18">
         <v>1.06</v>
       </c>
-      <c r="F6" s="25">
-        <v>0.64</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="23">
-        <v>6800</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" s="24">
-        <v>111618.7</v>
-      </c>
-      <c r="E7" s="25">
+      <c r="F10" s="18">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="16">
+        <v>2400</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="17">
+        <v>10865</v>
+      </c>
+      <c r="E11" s="18">
         <v>1.06</v>
       </c>
-      <c r="F7" s="25">
-        <v>0.67</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B8" s="23">
-        <v>14400</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" s="24">
-        <v>212003.3</v>
-      </c>
-      <c r="E8" s="25">
-        <v>1.06</v>
-      </c>
-      <c r="F8" s="25">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B9" s="23">
-        <v>5800</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="24">
-        <v>133612.6</v>
-      </c>
-      <c r="E9" s="25">
-        <v>1.06</v>
-      </c>
-      <c r="F9" s="25">
-        <v>0.56000000000000005</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B10" s="23">
-        <v>500</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D10" s="24">
-        <v>10727.7</v>
-      </c>
-      <c r="E10" s="25">
-        <v>1.06</v>
-      </c>
-      <c r="F10" s="25">
+      <c r="F11" s="18">
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B11" s="23">
-        <v>2400</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D11" s="24">
-        <v>10865</v>
-      </c>
-      <c r="E11" s="25">
-        <v>1.06</v>
-      </c>
-      <c r="F11" s="25">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
   </sheetData>
-  <phoneticPr fontId="9" type="noConversion"/>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -1965,7 +1761,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CAF5A36-638C-40FF-A541-E69329E36288}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1975,78 +1771,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>52</v>
+      <c r="A1" s="1" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B3" s="23">
+      <c r="A3" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="16">
         <f>SUMIF(MARCAS[CEBE],"GLOBAL",MARCAS[OBJ])</f>
         <v>42400</v>
       </c>
-      <c r="C3" s="25">
+      <c r="C3" s="18">
         <v>1.06</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B4" s="23">
+      <c r="A4" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" s="16">
         <f>MARCAS!B9*0.82</f>
         <v>4756</v>
       </c>
-      <c r="C4" s="25">
+      <c r="C4" s="18">
         <v>1.06</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B5" s="23">
+      <c r="A5" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="16">
         <f>+MARCAS!B8</f>
         <v>14400</v>
       </c>
-      <c r="C5" s="25">
+      <c r="C5" s="18">
         <v>1.06</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" s="23">
+      <c r="A6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="16">
         <f>MARCAS!B9*0.18</f>
         <v>1044</v>
       </c>
-      <c r="C6" s="25">
+      <c r="C6" s="18">
         <v>1.06</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B7" s="23">
+      <c r="A7" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="16">
         <f>+MARCAS!B11</f>
         <v>2400</v>
       </c>
-      <c r="C7" s="25">
+      <c r="C7" s="18">
         <v>1.06</v>
       </c>
     </row>
@@ -2058,7 +1854,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0490D270-0B83-4324-81C7-E84138AEEB58}">
   <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2070,369 +1866,423 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="8">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="B3" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="10">
+        <v>70</v>
+      </c>
+      <c r="D3" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="13">
+        <v>2</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="15">
+        <v>47</v>
+      </c>
+      <c r="D4" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="8">
+        <v>3</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="10">
+        <v>70</v>
+      </c>
+      <c r="D5" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="13">
+        <v>4</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="15">
+        <v>47</v>
+      </c>
+      <c r="D6" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="8">
         <v>5</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B7" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="10">
+        <v>60</v>
+      </c>
+      <c r="D7" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="13">
         <v>6</v>
       </c>
+      <c r="B8" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="15">
+        <v>60</v>
+      </c>
+      <c r="D8" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="8">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="10">
+        <v>60</v>
+      </c>
+      <c r="D9" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="13">
+        <v>9</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="15">
+        <v>60</v>
+      </c>
+      <c r="D10" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="8">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="10">
+        <v>60</v>
+      </c>
+      <c r="D11" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="13">
+        <v>11</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="15">
+        <v>70</v>
+      </c>
+      <c r="D12" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="8">
+        <v>13</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="10">
+        <v>47</v>
+      </c>
+      <c r="D13" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="13">
+        <v>14</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="15">
+        <v>70</v>
+      </c>
+      <c r="D14" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="8">
+        <v>15</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="10">
+        <v>70</v>
+      </c>
+      <c r="D15" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="13">
+        <v>19</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="15">
+        <v>60</v>
+      </c>
+      <c r="D16" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="8">
+        <v>22</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="10">
+        <v>60</v>
+      </c>
+      <c r="D17" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="13">
+        <v>23</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="15">
+        <v>60</v>
+      </c>
+      <c r="D18" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="8">
+        <v>24</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="10">
+        <v>70</v>
+      </c>
+      <c r="D19" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="13">
+        <v>25</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" s="15">
+        <v>70</v>
+      </c>
+      <c r="D20" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="8">
+        <v>28</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21" s="10">
+        <v>70</v>
+      </c>
+      <c r="D21" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="13">
+        <v>32</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="15">
+        <v>47</v>
+      </c>
+      <c r="D22" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="8">
+        <v>37</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C23" s="10">
+        <v>47</v>
+      </c>
+      <c r="D23" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="13">
+        <v>39</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" s="15">
+        <v>47</v>
+      </c>
+      <c r="D24" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="8">
+        <v>40</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C25" s="10">
+        <v>47</v>
+      </c>
+      <c r="D25" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="13">
+        <v>20</v>
+      </c>
+      <c r="B26" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C26" s="15">
+        <v>0</v>
+      </c>
+      <c r="D26" s="15"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="19">
+        <v>99</v>
+      </c>
+      <c r="B27" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="21">
+        <v>0</v>
+      </c>
+      <c r="D27" s="21"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CA3AA8D-30BC-4115-B13E-734CD6E68E67}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="C2" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="11">
-        <v>1</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="13">
-        <v>70</v>
-      </c>
-      <c r="D3" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="18">
-        <v>2</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="20">
-        <v>47</v>
-      </c>
-      <c r="D4" s="20">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="11">
-        <v>3</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="13">
-        <v>70</v>
-      </c>
-      <c r="D5" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="18">
-        <v>4</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="20">
-        <v>47</v>
-      </c>
-      <c r="D6" s="20">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="11">
-        <v>5</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="13">
-        <v>60</v>
-      </c>
-      <c r="D7" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="18">
-        <v>6</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="20">
-        <v>60</v>
-      </c>
-      <c r="D8" s="20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="11">
-        <v>8</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="13">
-        <v>60</v>
-      </c>
-      <c r="D9" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="18">
-        <v>9</v>
-      </c>
-      <c r="B10" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" s="20">
-        <v>60</v>
-      </c>
-      <c r="D10" s="20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="11">
-        <v>10</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="13">
-        <v>60</v>
-      </c>
-      <c r="D11" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="18">
-        <v>11</v>
-      </c>
-      <c r="B12" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="C12" s="20">
-        <v>70</v>
-      </c>
-      <c r="D12" s="20">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="11">
-        <v>13</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="13">
-        <v>47</v>
-      </c>
-      <c r="D13" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="18">
-        <v>14</v>
-      </c>
-      <c r="B14" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" s="20">
-        <v>70</v>
-      </c>
-      <c r="D14" s="20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="11">
-        <v>15</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="C15" s="13">
-        <v>70</v>
-      </c>
-      <c r="D15" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="18">
-        <v>19</v>
-      </c>
-      <c r="B16" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="C16" s="20">
-        <v>60</v>
-      </c>
-      <c r="D16" s="20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="11">
-        <v>22</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="C17" s="13">
-        <v>60</v>
-      </c>
-      <c r="D17" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="18">
-        <v>23</v>
-      </c>
-      <c r="B18" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="C18" s="20">
-        <v>60</v>
-      </c>
-      <c r="D18" s="20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="11">
-        <v>24</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" s="13">
-        <v>70</v>
-      </c>
-      <c r="D19" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="18">
-        <v>25</v>
-      </c>
-      <c r="B20" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="C20" s="20">
-        <v>70</v>
-      </c>
-      <c r="D20" s="20">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="11">
-        <v>28</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="C21" s="13">
-        <v>70</v>
-      </c>
-      <c r="D21" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="18">
-        <v>32</v>
-      </c>
-      <c r="B22" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="C22" s="20">
-        <v>47</v>
-      </c>
-      <c r="D22" s="20">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="11">
-        <v>37</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="C23" s="13">
-        <v>47</v>
-      </c>
-      <c r="D23" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="18">
-        <v>39</v>
-      </c>
-      <c r="B24" s="19" t="s">
-        <v>63</v>
-      </c>
-      <c r="C24" s="20">
-        <v>47</v>
-      </c>
-      <c r="D24" s="20">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="11">
-        <v>40</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="C25" s="13">
-        <v>47</v>
-      </c>
-      <c r="D25" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="18">
-        <v>20</v>
-      </c>
-      <c r="B26" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="C26" s="20">
-        <v>0</v>
-      </c>
-      <c r="D26" s="20"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="26">
-        <v>99</v>
-      </c>
-      <c r="B27" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="C27" s="28">
-        <v>0</v>
-      </c>
-      <c r="D27" s="28"/>
+        <v>300066580</v>
+      </c>
+      <c r="C3" s="12">
+        <v>46206</v>
+      </c>
+      <c r="D3" s="12">
+        <v>46256</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="11">
+        <v>300066581</v>
+      </c>
+      <c r="C4" s="12">
+        <v>46206</v>
+      </c>
+      <c r="D4" s="12">
+        <v>46256</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2443,106 +2293,52 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CA3AA8D-30BC-4115-B13E-734CD6E68E67}">
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="14">
-        <v>300066580</v>
-      </c>
-      <c r="C3" s="15">
-        <v>46206</v>
-      </c>
-      <c r="D3" s="15">
-        <v>46256</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="14">
-        <v>300066581</v>
-      </c>
-      <c r="C4" s="15">
-        <v>46206</v>
-      </c>
-      <c r="D4" s="15">
-        <v>46256</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{757B39EA-0E21-496B-AF3C-C43255427346}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>67</v>
+      <c r="A1" s="1" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>70</v>
+      <c r="A2" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B3" s="23">
+      <c r="A3" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" s="16">
         <v>490</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B4" s="23">
+      <c r="A4" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" s="16">
         <v>688</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="23">
+      <c r="A5" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" s="16">
         <v>1410</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B6" s="23">
+      <c r="A6" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B6" s="16">
         <v>2351</v>
       </c>
     </row>

</xml_diff>